<commit_message>
Add validity check to 3x3 GPS collection group
Update the relevance condition for the 'gps_pictures_3x3' group to
ensure it only triggers if a valid, non-empty plot ID has been
successfully matched (${plot_id} = ${plot_id_tmp}).

Previously, this group had an empty relevance condition, which could
cause it to unconditionally appear even if the enumerator entered an
invalid plot ID.
</commit_message>
<xml_diff>
--- a/kobo_management/forms/aGg4YcYHYyqKLiBfWPkjnA_260928.xlsx
+++ b/kobo_management/forms/aGg4YcYHYyqKLiBfWPkjnA_260928.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matteoramina/Documents/work/consulting/ci_ppc/ppc_data_pipeline/kobo_management/forms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDACC3A-D8D4-724C-910C-295DF4D5C336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E2FE84-010C-E04F-8EA2-B519F85DB714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="37600" yWindow="600" windowWidth="34560" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1926" uniqueCount="1122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1927" uniqueCount="1122">
   <si>
     <t>list_name</t>
   </si>
@@ -3875,152 +3875,152 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFBFBFBF"/>
+          <bgColor rgb="FFBFBFBF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF6D9E"/>
+          <bgColor rgb="FFFF6D9E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFD6E3BC"/>
           <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF6D9E"/>
-          <bgColor rgb="FFFF6D9E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4038,19 +4038,19 @@
       </font>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF6D9E"/>
-          <bgColor rgb="FFFF6D9E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <strike/>
       </font>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF6D9E"/>
+          <bgColor rgb="FFFF6D9E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <strike/>
       </font>
@@ -4364,112 +4364,112 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFE4E300"/>
           <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4497,6 +4497,62 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFDCC97A"/>
           <bgColor rgb="FFDCC97A"/>
         </patternFill>
@@ -4537,6 +4593,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFABF8F"/>
           <bgColor rgb="FFFABF8F"/>
         </patternFill>
@@ -4553,6 +4617,78 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFB8CCE4"/>
           <bgColor rgb="FFB8CCE4"/>
         </patternFill>
@@ -4561,6 +4697,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFEEB400"/>
           <bgColor rgb="FFEEB400"/>
         </patternFill>
@@ -4577,6 +4721,30 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFC2D69B"/>
           <bgColor rgb="FFC2D69B"/>
         </patternFill>
@@ -4585,6 +4753,78 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFF9900"/>
           <bgColor rgb="FFFF9900"/>
         </patternFill>
@@ -4593,6 +4833,158 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FF4685D2"/>
           <bgColor rgb="FF4685D2"/>
         </patternFill>
@@ -4609,6 +5001,110 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFF9900"/>
           <bgColor rgb="FFFF9900"/>
         </patternFill>
@@ -4617,16 +5113,40 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4641,38 +5161,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFFF9900"/>
           <bgColor rgb="FFFF9900"/>
         </patternFill>
@@ -4681,496 +5169,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFFABF8F"/>
           <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5221,8 +5221,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5242,8 +5242,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6013,6 +6013,38 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFF0000"/>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
@@ -6021,6 +6053,46 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFD6E3BC"/>
           <bgColor rgb="FFD6E3BC"/>
         </patternFill>
@@ -6029,6 +6101,70 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFABF8F"/>
           <bgColor rgb="FFFABF8F"/>
         </patternFill>
@@ -6037,6 +6173,70 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFC2D69B"/>
           <bgColor rgb="FFC2D69B"/>
         </patternFill>
@@ -6053,6 +6253,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFDCC97A"/>
           <bgColor rgb="FFDCC97A"/>
         </patternFill>
@@ -6061,6 +6269,150 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFE4E300"/>
           <bgColor rgb="FFE4E300"/>
         </patternFill>
@@ -6069,32 +6421,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6109,6 +6437,38 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFF9900"/>
           <bgColor rgb="FFFF9900"/>
         </patternFill>
@@ -6117,14 +6477,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFB8CCE4"/>
           <bgColor rgb="FFB8CCE4"/>
         </patternFill>
@@ -6141,352 +6493,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
+          <fgColor rgb="FFFF6D9E"/>
+          <bgColor rgb="FFFF6D9E"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6496,14 +6504,6 @@
       </font>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF6D9E"/>
-          <bgColor rgb="FFFF6D9E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <strike/>
       </font>
@@ -6511,6 +6511,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFF9900"/>
           <bgColor rgb="FFFF9900"/>
         </patternFill>
@@ -6519,6 +6527,70 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFBFBFBF"/>
+          <bgColor rgb="FFBFBFBF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF6D9E"/>
+          <bgColor rgb="FFFF6D9E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFF2F2F2"/>
           <bgColor rgb="FFF2F2F2"/>
         </patternFill>
@@ -6527,6 +6599,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFB8CCE4"/>
           <bgColor rgb="FFB8CCE4"/>
         </patternFill>
@@ -6543,6 +6623,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFC2D69B"/>
           <bgColor rgb="FFC2D69B"/>
         </patternFill>
@@ -6575,6 +6663,206 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFB2A1C7"/>
           <bgColor rgb="FFB2A1C7"/>
         </patternFill>
@@ -6583,6 +6871,70 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFF9900"/>
           <bgColor rgb="FFFF9900"/>
         </patternFill>
@@ -6591,24 +6943,96 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
+          <fgColor rgb="FFFF6D9E"/>
+          <bgColor rgb="FFFF6D9E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9E004F"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6617,430 +7041,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFBFBFBF"/>
           <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF6D9E"/>
-          <bgColor rgb="FFFF6D9E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9E004F"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF6D9E"/>
-          <bgColor rgb="FFFF6D9E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
         </patternFill>
       </fill>
     </dxf>
@@ -12434,7 +12434,9 @@
       <c r="M122" s="1"/>
       <c r="N122" s="1"/>
       <c r="O122" s="1"/>
-      <c r="P122" s="1"/>
+      <c r="P122" s="1" t="s">
+        <v>318</v>
+      </c>
       <c r="Q122" s="1"/>
       <c r="R122" s="1"/>
       <c r="S122" s="1"/>
@@ -16686,37 +16688,37 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:X236">
     <cfRule type="expression" dxfId="403" priority="374" stopIfTrue="1">
+      <formula>$A1="comments"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="402" priority="374" stopIfTrue="1">
       <formula>OR($A1="geopoint", $A1="geoshape", $A1="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="402" priority="374" stopIfTrue="1">
-      <formula>OR($A1="audio audit", $A1="text audit", $A1="speed violations count", $A1="speed violations list", $A1="speed violations audit")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="401" priority="420" stopIfTrue="1">
       <formula>$A1="note"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="400" priority="374" stopIfTrue="1">
-      <formula>$A1="comments"</formula>
+      <formula>$A1="image"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="399" priority="374" stopIfTrue="1">
-      <formula>$A1="text"</formula>
+      <formula>$A1="barcode"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="398" priority="374" stopIfTrue="1">
-      <formula>OR($A1="calculate", $A1="calculate_here")</formula>
+      <formula>OR($A1="username", $A1="phonenumber", $A1="start", $A1="end", $A1="deviceid", $A1="subscriberid", $A1="simserial", $A1="caseid")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="397" priority="374" stopIfTrue="1">
-      <formula>$A1="end group"</formula>
+      <formula>OR($A1="audio audit", $A1="text audit", $A1="speed violations count", $A1="speed violations list", $A1="speed violations audit")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="396" priority="374" stopIfTrue="1">
-      <formula>$A1="barcode"</formula>
+      <formula>OR(AND(LEFT($A1, 16)="select_multiple ", LEN($A1)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1, 17)))), AND(LEFT($A1, 11)="select_one ", LEN($A1)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1, 12)))))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="395" priority="374" stopIfTrue="1">
-      <formula>$A1="note"</formula>
+      <formula>$A1="end repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="394" priority="374" stopIfTrue="1">
-      <formula>$A1="begin group"</formula>
+      <formula>$A1="integer"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="393" priority="374" stopIfTrue="1">
-      <formula>$A1="decimal"</formula>
+      <formula>OR($A1="audio", $A1="video")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="392" priority="374" stopIfTrue="1">
       <formula>OR($A1="date", $A1="datetime")</formula>
@@ -16725,25 +16727,25 @@
       <formula>OR(AND(LEFT($A1, 14)="sensor_stream ", LEN($A1)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1, 15)))), AND(LEFT($A1, 17)="sensor_statistic ", LEN($A1)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1, 18)))))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="390" priority="374" stopIfTrue="1">
-      <formula>OR($A1="audio", $A1="video")</formula>
+      <formula>$A1="begin repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="389" priority="374" stopIfTrue="1">
-      <formula>OR($A1="username", $A1="phonenumber", $A1="start", $A1="end", $A1="deviceid", $A1="subscriberid", $A1="simserial", $A1="caseid")</formula>
+      <formula>$A1="decimal"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="388" priority="374" stopIfTrue="1">
-      <formula>$A1="begin repeat"</formula>
+      <formula>$A1="begin group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="387" priority="374" stopIfTrue="1">
-      <formula>$A1="image"</formula>
+      <formula>$A1="note"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="386" priority="374" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1, 16)="select_multiple ", LEN($A1)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1, 17)))), AND(LEFT($A1, 11)="select_one ", LEN($A1)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1, 12)))))</formula>
+      <formula>$A1="end group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="385" priority="374" stopIfTrue="1">
-      <formula>$A1="end repeat"</formula>
+      <formula>OR($A1="calculate", $A1="calculate_here")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="384" priority="374" stopIfTrue="1">
-      <formula>$A1="integer"</formula>
+      <formula>$A1="text"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A8:X11 A18:X18 A24:X25 A28:X28">
@@ -16754,21 +16756,21 @@
       <formula>$A8="note"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="381" priority="404" stopIfTrue="1">
+      <formula>OR($A8="date", $A8="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="380" priority="404" stopIfTrue="1">
+      <formula>$A8="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="379" priority="404" stopIfTrue="1">
+      <formula>$A8="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="378" priority="404" stopIfTrue="1">
       <formula>OR($A8="audio", $A8="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="380" priority="404" stopIfTrue="1">
-      <formula>OR($A8="date", $A8="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="379" priority="404" stopIfTrue="1">
-      <formula>$A8="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="378" priority="404" stopIfTrue="1">
-      <formula>$A8="barcode"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A8:X11 A18:X18 A24:X25">
     <cfRule type="expression" dxfId="377" priority="394" stopIfTrue="1">
-      <formula>$A8="integer"</formula>
+      <formula>$A8="end group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="376" priority="394" stopIfTrue="1">
       <formula>$A8="text"</formula>
@@ -16777,122 +16779,122 @@
       <formula>OR($A8="geopoint", $A8="geoshape", $A8="geotrace")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="374" priority="394" stopIfTrue="1">
+      <formula>$A8="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="373" priority="394" stopIfTrue="1">
+      <formula>OR($A8="username", $A8="phonenumber", $A8="start", $A8="end", $A8="deviceid", $A8="subscriberid", $A8="simserial", $A8="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="372" priority="394" stopIfTrue="1">
+      <formula>$A8="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="371" priority="394" stopIfTrue="1">
+      <formula>$A8="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="370" priority="394" stopIfTrue="1">
+      <formula>$A8="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="369" priority="394" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A8, 16)="select_multiple ", LEN($A8)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A8, 17)))), AND(LEFT($A8, 11)="select_one ", LEN($A8)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A8, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="368" priority="394" stopIfTrue="1">
+      <formula>OR($A8="audio audit", $A8="text audit", $A8="speed violations count", $A8="speed violations list", $A8="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="367" priority="394" stopIfTrue="1">
       <formula>$A8="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="373" priority="394" stopIfTrue="1">
-      <formula>OR($A8="audio audit", $A8="text audit", $A8="speed violations count", $A8="speed violations list", $A8="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="372" priority="394" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A8, 16)="select_multiple ", LEN($A8)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A8, 17)))), AND(LEFT($A8, 11)="select_one ", LEN($A8)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A8, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="371" priority="394" stopIfTrue="1">
-      <formula>$A8="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="370" priority="394" stopIfTrue="1">
-      <formula>$A8="end repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="369" priority="394" stopIfTrue="1">
-      <formula>$A8="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="368" priority="394" stopIfTrue="1">
-      <formula>$A8="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="367" priority="394" stopIfTrue="1">
-      <formula>OR($A8="username", $A8="phonenumber", $A8="start", $A8="end", $A8="deviceid", $A8="subscriberid", $A8="simserial", $A8="caseid")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A28:X28">
     <cfRule type="expression" dxfId="366" priority="346" stopIfTrue="1">
+      <formula>OR($A28="geopoint", $A28="geoshape", $A28="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="365" priority="346" stopIfTrue="1">
+      <formula>$A28="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="364" priority="346" stopIfTrue="1">
+      <formula>$A28="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="363" priority="346" stopIfTrue="1">
+      <formula>OR($A28="audio audit", $A28="text audit", $A28="speed violations count", $A28="speed violations list", $A28="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="362" priority="346" stopIfTrue="1">
+      <formula>$A28="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="361" priority="346" stopIfTrue="1">
+      <formula>OR($A28="username", $A28="phonenumber", $A28="start", $A28="end", $A28="deviceid", $A28="subscriberid", $A28="simserial", $A28="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="360" priority="346" stopIfTrue="1">
       <formula>$A28="begin repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="365" priority="346" stopIfTrue="1">
+    <cfRule type="expression" dxfId="359" priority="346" stopIfTrue="1">
       <formula>OR(AND(LEFT($A28, 16)="select_multiple ", LEN($A28)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A28, 17)))), AND(LEFT($A28, 11)="select_one ", LEN($A28)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A28, 12)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="364" priority="346" stopIfTrue="1">
+    <cfRule type="expression" dxfId="358" priority="346" stopIfTrue="1">
       <formula>$A28="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="363" priority="346" stopIfTrue="1">
+    <cfRule type="expression" dxfId="357" priority="346" stopIfTrue="1">
       <formula>$A28="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="362" priority="346" stopIfTrue="1">
+    <cfRule type="expression" dxfId="356" priority="346" stopIfTrue="1">
       <formula>$A28="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="361" priority="346" stopIfTrue="1">
-      <formula>$A28="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="360" priority="346" stopIfTrue="1">
-      <formula>$A28="end repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="359" priority="346" stopIfTrue="1">
-      <formula>OR($A28="geopoint", $A28="geoshape", $A28="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="358" priority="346" stopIfTrue="1">
-      <formula>OR($A28="username", $A28="phonenumber", $A28="start", $A28="end", $A28="deviceid", $A28="subscriberid", $A28="simserial", $A28="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="357" priority="346" stopIfTrue="1">
-      <formula>OR($A28="audio audit", $A28="text audit", $A28="speed violations count", $A28="speed violations list", $A28="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="356" priority="346" stopIfTrue="1">
-      <formula>$A28="end group"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A35:X35 C39">
     <cfRule type="expression" dxfId="355" priority="262" stopIfTrue="1">
+      <formula>OR($A35="audio", $A35="video")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="354" priority="262" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A35, 16)="select_multiple ", LEN($A35)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A35, 17)))), AND(LEFT($A35, 11)="select_one ", LEN($A35)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A35, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="353" priority="262" stopIfTrue="1">
+      <formula>$A35="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="352" priority="262" stopIfTrue="1">
+      <formula>$A35="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="351" priority="262" stopIfTrue="1">
+      <formula>$A35="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="350" priority="262" stopIfTrue="1">
+      <formula>$A35="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="349" priority="262" stopIfTrue="1">
+      <formula>$A35="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="348" priority="262" stopIfTrue="1">
+      <formula>OR($A35="geopoint", $A35="geoshape", $A35="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="347" priority="262" stopIfTrue="1">
+      <formula>OR($A35="username", $A35="phonenumber", $A35="start", $A35="end", $A35="deviceid", $A35="subscriberid", $A35="simserial", $A35="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="346" priority="262" stopIfTrue="1">
+      <formula>$A35="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="345" priority="262" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A35, 14)="sensor_stream ", LEN($A35)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A35, 15)))), AND(LEFT($A35, 17)="sensor_statistic ", LEN($A35)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A35, 18)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="344" priority="262" stopIfTrue="1">
+      <formula>$A35="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="343" priority="262" stopIfTrue="1">
+      <formula>$A35="comments"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="342" priority="262" stopIfTrue="1">
+      <formula>$A35="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="341" priority="262" stopIfTrue="1">
+      <formula>$A35="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="340" priority="262" stopIfTrue="1">
+      <formula>OR($A35="calculate", $A35="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="339" priority="262" stopIfTrue="1">
       <formula>OR($A35="audio audit", $A35="text audit", $A35="speed violations count", $A35="speed violations list", $A35="speed violations audit")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="354" priority="262" stopIfTrue="1">
-      <formula>OR($A35="geopoint", $A35="geoshape", $A35="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="353" priority="262" stopIfTrue="1">
-      <formula>$A35="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="352" priority="262" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A35, 14)="sensor_stream ", LEN($A35)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A35, 15)))), AND(LEFT($A35, 17)="sensor_statistic ", LEN($A35)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A35, 18)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="351" priority="262" stopIfTrue="1">
-      <formula>$A35="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="350" priority="262" stopIfTrue="1">
-      <formula>$A35="comments"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="349" priority="262" stopIfTrue="1">
-      <formula>$A35="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="348" priority="262" stopIfTrue="1">
-      <formula>OR($A35="calculate", $A35="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="347" priority="262" stopIfTrue="1">
-      <formula>$A35="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="346" priority="262" stopIfTrue="1">
+    <cfRule type="expression" dxfId="338" priority="262" stopIfTrue="1">
       <formula>$A35="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="345" priority="262" stopIfTrue="1">
+    <cfRule type="expression" dxfId="337" priority="262" stopIfTrue="1">
       <formula>OR($A35="date", $A35="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="344" priority="262" stopIfTrue="1">
-      <formula>OR($A35="audio", $A35="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="343" priority="262" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A35, 16)="select_multiple ", LEN($A35)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A35, 17)))), AND(LEFT($A35, 11)="select_one ", LEN($A35)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A35, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="342" priority="262" stopIfTrue="1">
-      <formula>$A35="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="341" priority="262" stopIfTrue="1">
-      <formula>$A35="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="340" priority="262" stopIfTrue="1">
-      <formula>$A35="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="339" priority="262" stopIfTrue="1">
-      <formula>$A35="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="338" priority="262" stopIfTrue="1">
-      <formula>OR($A35="username", $A35="phonenumber", $A35="start", $A35="end", $A35="deviceid", $A35="subscriberid", $A35="simserial", $A35="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="337" priority="262" stopIfTrue="1">
-      <formula>$A35="begin repeat"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B236 V10:W236">
@@ -16901,114 +16903,114 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C236">
-    <cfRule type="expression" dxfId="335" priority="343" stopIfTrue="1">
+    <cfRule type="expression" dxfId="335" priority="343">
+      <formula>#REF!="false"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="334" priority="343" stopIfTrue="1">
       <formula>OR(AND(LEFT($A1, 14)="sensor_stream ", LEN($A1)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1, 15)))), AND(LEFT($A1, 17)="sensor_statistic ", LEN($A1)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1, 18)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="334" priority="343">
-      <formula>#REF!="false"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C12">
     <cfRule type="expression" dxfId="333" priority="326" stopIfTrue="1">
+      <formula>OR($A12="audio audit", $A12="text audit", $A12="speed violations count", $A12="speed violations list", $A12="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="332" priority="326" stopIfTrue="1">
+      <formula>$A12="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="331" priority="326" stopIfTrue="1">
+      <formula>$A12="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="330" priority="326" stopIfTrue="1">
       <formula>$A12="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="332" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="329" priority="326" stopIfTrue="1">
       <formula>$A12="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="331" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="328" priority="326" stopIfTrue="1">
       <formula>$A12="decimal"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="330" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="327" priority="326" stopIfTrue="1">
       <formula>OR(AND(LEFT($A12, 16)="select_multiple ", LEN($A12)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A12, 17)))), AND(LEFT($A12, 11)="select_one ", LEN($A12)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A12, 12)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="329" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="326" priority="326" stopIfTrue="1">
+      <formula>$A12="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="325" priority="326" stopIfTrue="1">
       <formula>$A12="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="328" priority="326" stopIfTrue="1">
-      <formula>$A12="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="327" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="324" priority="326" stopIfTrue="1">
       <formula>OR($A12="calculate", $A12="calculate_here")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="326" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="323" priority="326" stopIfTrue="1">
       <formula>$A12="image"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="325" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="322" priority="326" stopIfTrue="1">
       <formula>OR($A12="username", $A12="phonenumber", $A12="start", $A12="end", $A12="deviceid", $A12="subscriberid", $A12="simserial", $A12="caseid")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="324" priority="326" stopIfTrue="1">
-      <formula>OR($A12="audio audit", $A12="text audit", $A12="speed violations count", $A12="speed violations list", $A12="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="323" priority="326" stopIfTrue="1">
-      <formula>$A12="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="322" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="321" priority="326" stopIfTrue="1">
       <formula>$A12="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="321" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="320" priority="326" stopIfTrue="1">
       <formula>OR($A12="geopoint", $A12="geoshape", $A12="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="320" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="319" priority="326" stopIfTrue="1">
       <formula>$A12="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="319" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="318" priority="326" stopIfTrue="1">
       <formula>OR($A12="date", $A12="datetime")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="318" priority="326" stopIfTrue="1">
+    <cfRule type="expression" dxfId="317" priority="326" stopIfTrue="1">
       <formula>OR($A12="audio", $A12="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="317" priority="326" stopIfTrue="1">
-      <formula>$A12="end group"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18 C24:C25 C28:C30">
     <cfRule type="expression" dxfId="316" priority="310" stopIfTrue="1">
-      <formula>OR($A18="username", $A18="phonenumber", $A18="start", $A18="end", $A18="deviceid", $A18="subscriberid", $A18="simserial", $A18="caseid")</formula>
+      <formula>$A18="text"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="315" priority="310" stopIfTrue="1">
-      <formula>$A18="begin repeat"</formula>
+      <formula>$A18="end repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="314" priority="310" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A18, 16)="select_multiple ", LEN($A18)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A18, 17)))), AND(LEFT($A18, 11)="select_one ", LEN($A18)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A18, 12)))))</formula>
+      <formula>OR($A18="geopoint", $A18="geoshape", $A18="geotrace")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="313" priority="310" stopIfTrue="1">
       <formula>OR($A18="audio audit", $A18="text audit", $A18="speed violations count", $A18="speed violations list", $A18="speed violations audit")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="312" priority="310" stopIfTrue="1">
-      <formula>OR($A18="geopoint", $A18="geoshape", $A18="geotrace")</formula>
+      <formula>OR(AND(LEFT($A18, 16)="select_multiple ", LEN($A18)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A18, 17)))), AND(LEFT($A18, 11)="select_one ", LEN($A18)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A18, 12)))))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="311" priority="310" stopIfTrue="1">
-      <formula>$A18="image"</formula>
+      <formula>$A18="begin repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="310" priority="310" stopIfTrue="1">
-      <formula>$A18="barcode"</formula>
+      <formula>OR($A18="username", $A18="phonenumber", $A18="start", $A18="end", $A18="deviceid", $A18="subscriberid", $A18="simserial", $A18="caseid")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="309" priority="310" stopIfTrue="1">
-      <formula>$A18="end group"</formula>
+      <formula>OR($A18="date", $A18="datetime")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="308" priority="310" stopIfTrue="1">
-      <formula>OR($A18="calculate", $A18="calculate_here")</formula>
+      <formula>$A18="integer"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="307" priority="310" stopIfTrue="1">
-      <formula>$A18="note"</formula>
+      <formula>$A18="begin group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="306" priority="310" stopIfTrue="1">
       <formula>$A18="decimal"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="305" priority="310" stopIfTrue="1">
-      <formula>$A18="begin group"</formula>
+      <formula>$A18="note"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="304" priority="310" stopIfTrue="1">
-      <formula>$A18="integer"</formula>
+      <formula>OR($A18="calculate", $A18="calculate_here")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="303" priority="310" stopIfTrue="1">
-      <formula>OR($A18="date", $A18="datetime")</formula>
+      <formula>$A18="end group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="302" priority="310" stopIfTrue="1">
-      <formula>$A18="end repeat"</formula>
+      <formula>$A18="barcode"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="301" priority="310" stopIfTrue="1">
-      <formula>$A18="text"</formula>
+      <formula>$A18="image"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C30 C18 C24:C25">
@@ -17018,34 +17020,34 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C30">
     <cfRule type="expression" dxfId="299" priority="298" stopIfTrue="1">
+      <formula>$A28="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="298" priority="298" stopIfTrue="1">
+      <formula>$A28="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="297" priority="298" stopIfTrue="1">
+      <formula>$A28="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="296" priority="298" stopIfTrue="1">
+      <formula>OR($A28="username", $A28="phonenumber", $A28="start", $A28="end", $A28="deviceid", $A28="subscriberid", $A28="simserial", $A28="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="295" priority="298" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A28, 16)="select_multiple ", LEN($A28)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A28, 17)))), AND(LEFT($A28, 11)="select_one ", LEN($A28)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A28, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="294" priority="298" stopIfTrue="1">
+      <formula>$A28="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="293" priority="298" stopIfTrue="1">
+      <formula>$A28="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="292" priority="298" stopIfTrue="1">
+      <formula>$A28="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="291" priority="298" stopIfTrue="1">
+      <formula>OR($A28="geopoint", $A28="geoshape", $A28="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="290" priority="298" stopIfTrue="1">
       <formula>$A28="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="298" priority="298" stopIfTrue="1">
-      <formula>OR($A28="geopoint", $A28="geoshape", $A28="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="297" priority="298" stopIfTrue="1">
-      <formula>$A28="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="296" priority="298" stopIfTrue="1">
-      <formula>$A28="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="295" priority="298" stopIfTrue="1">
-      <formula>$A28="end repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="294" priority="298" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A28, 16)="select_multiple ", LEN($A28)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A28, 17)))), AND(LEFT($A28, 11)="select_one ", LEN($A28)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A28, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="293" priority="298" stopIfTrue="1">
-      <formula>OR($A28="username", $A28="phonenumber", $A28="start", $A28="end", $A28="deviceid", $A28="subscriberid", $A28="simserial", $A28="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="292" priority="298" stopIfTrue="1">
-      <formula>$A28="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="291" priority="298" stopIfTrue="1">
-      <formula>$A28="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="290" priority="298" stopIfTrue="1">
-      <formula>$A28="integer"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="289" priority="298" stopIfTrue="1">
       <formula>OR($A28="audio audit", $A28="text audit", $A28="speed violations count", $A28="speed violations list", $A28="speed violations audit")</formula>
@@ -17053,49 +17055,49 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="C29:C30">
     <cfRule type="expression" dxfId="288" priority="281" stopIfTrue="1">
+      <formula>OR($A29="username", $A29="phonenumber", $A29="start", $A29="end", $A29="deviceid", $A29="subscriberid", $A29="simserial", $A29="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="287" priority="281" stopIfTrue="1">
+      <formula>OR($A29="date", $A29="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="286" priority="281" stopIfTrue="1">
+      <formula>OR($A29="audio", $A29="video")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="285" priority="281" stopIfTrue="1">
+      <formula>OR($A29="geopoint", $A29="geoshape", $A29="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="284" priority="281" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A29, 16)="select_multiple ", LEN($A29)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A29, 17)))), AND(LEFT($A29, 11)="select_one ", LEN($A29)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A29, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="283" priority="281" stopIfTrue="1">
+      <formula>$A29="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="282" priority="281" stopIfTrue="1">
+      <formula>$A29="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="281" priority="281" stopIfTrue="1">
+      <formula>$A29="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="280" priority="281" stopIfTrue="1">
+      <formula>$A29="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="279" priority="281" stopIfTrue="1">
+      <formula>OR($A29="calculate", $A29="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="278" priority="281" stopIfTrue="1">
+      <formula>OR($A29="audio audit", $A29="text audit", $A29="speed violations count", $A29="speed violations list", $A29="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="277" priority="281" stopIfTrue="1">
+      <formula>$A29="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="276" priority="281" stopIfTrue="1">
+      <formula>$A29="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="275" priority="281" stopIfTrue="1">
+      <formula>$A29="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="274" priority="281" stopIfTrue="1">
       <formula>$A29="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="287" priority="281" stopIfTrue="1">
-      <formula>$A29="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="286" priority="281" stopIfTrue="1">
-      <formula>$A29="end repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="285" priority="281" stopIfTrue="1">
-      <formula>$A29="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="284" priority="281" stopIfTrue="1">
-      <formula>OR($A29="date", $A29="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="283" priority="281" stopIfTrue="1">
-      <formula>OR($A29="audio", $A29="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="282" priority="281" stopIfTrue="1">
-      <formula>OR($A29="username", $A29="phonenumber", $A29="start", $A29="end", $A29="deviceid", $A29="subscriberid", $A29="simserial", $A29="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="281" priority="281" stopIfTrue="1">
-      <formula>OR($A29="geopoint", $A29="geoshape", $A29="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="280" priority="281" stopIfTrue="1">
-      <formula>OR($A29="calculate", $A29="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="279" priority="281" stopIfTrue="1">
-      <formula>$A29="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="278" priority="281" stopIfTrue="1">
-      <formula>$A29="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="277" priority="281" stopIfTrue="1">
-      <formula>$A29="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="276" priority="281" stopIfTrue="1">
-      <formula>$A29="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="275" priority="281" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A29, 16)="select_multiple ", LEN($A29)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A29, 17)))), AND(LEFT($A29, 11)="select_one ", LEN($A29)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A29, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="274" priority="281" stopIfTrue="1">
-      <formula>OR($A29="audio audit", $A29="text audit", $A29="speed violations count", $A29="speed violations list", $A29="speed violations audit")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="273" priority="281" stopIfTrue="1">
       <formula>$A29="begin repeat"</formula>
@@ -17412,7 +17414,7 @@
       <formula>OR($A221="geopoint", $A221="geoshape", $A221="geotrace")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="175" priority="418" stopIfTrue="1">
-      <formula>$A221="begin repeat"</formula>
+      <formula>OR($A221="audio", $A221="video")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="174" priority="409" stopIfTrue="1">
       <formula>$A221="decimal"</formula>
@@ -17421,7 +17423,7 @@
       <formula>AL221="false"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="172" priority="418" stopIfTrue="1">
-      <formula>OR($A221="audio", $A221="video")</formula>
+      <formula>$A221="begin repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="171" priority="391" stopIfTrue="1">
       <formula>$A221="barcode"</formula>
@@ -17455,55 +17457,55 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="Q148:W151">
     <cfRule type="expression" dxfId="164" priority="226" stopIfTrue="1">
+      <formula>$A148="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="163" priority="226" stopIfTrue="1">
+      <formula>$A148="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="162" priority="226" stopIfTrue="1">
+      <formula>$A148="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="161" priority="226" stopIfTrue="1">
+      <formula>$A148="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="160" priority="226" stopIfTrue="1">
+      <formula>OR($A148="date", $A148="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="159" priority="226" stopIfTrue="1">
+      <formula>$A148="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="158" priority="226" stopIfTrue="1">
+      <formula>$A148="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="157" priority="226" stopIfTrue="1">
+      <formula>$A148="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="156" priority="226" stopIfTrue="1">
+      <formula>$A148="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="155" priority="226" stopIfTrue="1">
+      <formula>OR($A148="calculate", $A148="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="154" priority="226" stopIfTrue="1">
+      <formula>OR($A148="audio audit", $A148="text audit", $A148="speed violations count", $A148="speed violations list", $A148="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="153" priority="226" stopIfTrue="1">
+      <formula>OR($A148="username", $A148="phonenumber", $A148="start", $A148="end", $A148="deviceid", $A148="subscriberid", $A148="simserial", $A148="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="152" priority="226" stopIfTrue="1">
       <formula>OR(AND(LEFT($A148, 16)="select_multiple ", LEN($A148)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A148, 17)))), AND(LEFT($A148, 11)="select_one ", LEN($A148)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A148, 12)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="163" priority="226" stopIfTrue="1">
-      <formula>$A148="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="162" priority="226" stopIfTrue="1">
-      <formula>OR($A148="audio", $A148="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="161" priority="226" stopIfTrue="1">
-      <formula>$A148="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="160" priority="226" stopIfTrue="1">
+    <cfRule type="expression" dxfId="151" priority="226" stopIfTrue="1">
       <formula>OR($A148="geopoint", $A148="geoshape", $A148="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="159" priority="226" stopIfTrue="1">
-      <formula>$A148="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="158" priority="226" stopIfTrue="1">
-      <formula>$A148="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="157" priority="226" stopIfTrue="1">
-      <formula>$A148="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="156" priority="226" stopIfTrue="1">
-      <formula>$A148="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="155" priority="226" stopIfTrue="1">
-      <formula>$A148="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="154" priority="226" stopIfTrue="1">
-      <formula>OR($A148="date", $A148="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="153" priority="226" stopIfTrue="1">
-      <formula>$A148="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="152" priority="226" stopIfTrue="1">
-      <formula>OR($A148="calculate", $A148="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="151" priority="226" stopIfTrue="1">
-      <formula>OR($A148="username", $A148="phonenumber", $A148="start", $A148="end", $A148="deviceid", $A148="subscriberid", $A148="simserial", $A148="caseid")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="150" priority="226" stopIfTrue="1">
       <formula>$A148="integer"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="149" priority="226" stopIfTrue="1">
-      <formula>OR($A148="audio audit", $A148="text audit", $A148="speed violations count", $A148="speed violations list", $A148="speed violations audit")</formula>
+      <formula>OR($A148="audio", $A148="video")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="148" priority="226" stopIfTrue="1">
-      <formula>$A148="end repeat"</formula>
+      <formula>$A148="decimal"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q169:W172">
@@ -17532,190 +17534,190 @@
       <formula>$A169="text"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="139" priority="209" stopIfTrue="1">
-      <formula>$A169="integer"</formula>
+      <formula>$A169="note"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="138" priority="209" stopIfTrue="1">
-      <formula>$A169="begin group"</formula>
+      <formula>$A169="barcode"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="137" priority="209" stopIfTrue="1">
-      <formula>OR($A169="username", $A169="phonenumber", $A169="start", $A169="end", $A169="deviceid", $A169="subscriberid", $A169="simserial", $A169="caseid")</formula>
+      <formula>$A169="end repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="136" priority="209" stopIfTrue="1">
-      <formula>OR($A169="date", $A169="datetime")</formula>
+      <formula>$A169="begin repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="135" priority="209" stopIfTrue="1">
       <formula>$A169="end group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="134" priority="209" stopIfTrue="1">
-      <formula>$A169="begin repeat"</formula>
+      <formula>$A169="integer"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="133" priority="209" stopIfTrue="1">
-      <formula>$A169="end repeat"</formula>
+      <formula>$A169="begin group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="132" priority="209" stopIfTrue="1">
-      <formula>$A169="barcode"</formula>
+      <formula>OR($A169="username", $A169="phonenumber", $A169="start", $A169="end", $A169="deviceid", $A169="subscriberid", $A169="simserial", $A169="caseid")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="131" priority="209" stopIfTrue="1">
-      <formula>$A169="note"</formula>
+      <formula>OR($A169="date", $A169="datetime")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q186:W189">
     <cfRule type="expression" dxfId="130" priority="192" stopIfTrue="1">
-      <formula>$A186="note"</formula>
+      <formula>OR($A186="date", $A186="datetime")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="129" priority="192" stopIfTrue="1">
-      <formula>OR($A186="audio audit", $A186="text audit", $A186="speed violations count", $A186="speed violations list", $A186="speed violations audit")</formula>
+      <formula>OR($A186="calculate", $A186="calculate_here")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="128" priority="192" stopIfTrue="1">
+      <formula>OR($A186="geopoint", $A186="geoshape", $A186="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="127" priority="192" stopIfTrue="1">
+      <formula>$A186="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="126" priority="192" stopIfTrue="1">
       <formula>$A186="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="127" priority="192" stopIfTrue="1">
-      <formula>OR($A186="calculate", $A186="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="126" priority="192" stopIfTrue="1">
-      <formula>OR($A186="date", $A186="datetime")</formula>
-    </cfRule>
     <cfRule type="expression" dxfId="125" priority="192" stopIfTrue="1">
-      <formula>OR($A186="geopoint", $A186="geoshape", $A186="geotrace")</formula>
+      <formula>$A186="integer"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="124" priority="192" stopIfTrue="1">
-      <formula>$A186="begin group"</formula>
+      <formula>OR($A186="username", $A186="phonenumber", $A186="start", $A186="end", $A186="deviceid", $A186="subscriberid", $A186="simserial", $A186="caseid")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="123" priority="192" stopIfTrue="1">
-      <formula>$A186="end group"</formula>
+      <formula>OR(AND(LEFT($A186, 16)="select_multiple ", LEN($A186)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A186, 17)))), AND(LEFT($A186, 11)="select_one ", LEN($A186)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A186, 12)))))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="122" priority="192" stopIfTrue="1">
-      <formula>$A186="decimal"</formula>
+      <formula>$A186="end repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="121" priority="192" stopIfTrue="1">
-      <formula>OR($A186="audio", $A186="video")</formula>
+      <formula>$A186="begin repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="120" priority="192" stopIfTrue="1">
       <formula>$A186="image"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="119" priority="192" stopIfTrue="1">
-      <formula>$A186="begin repeat"</formula>
+      <formula>OR($A186="audio", $A186="video")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="118" priority="192" stopIfTrue="1">
-      <formula>$A186="end repeat"</formula>
+      <formula>$A186="decimal"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="117" priority="192" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A186, 16)="select_multiple ", LEN($A186)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A186, 17)))), AND(LEFT($A186, 11)="select_one ", LEN($A186)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A186, 12)))))</formula>
+      <formula>$A186="begin group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="116" priority="192" stopIfTrue="1">
-      <formula>OR($A186="username", $A186="phonenumber", $A186="start", $A186="end", $A186="deviceid", $A186="subscriberid", $A186="simserial", $A186="caseid")</formula>
+      <formula>$A186="end group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="115" priority="192" stopIfTrue="1">
-      <formula>$A186="integer"</formula>
+      <formula>$A186="note"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="114" priority="192" stopIfTrue="1">
-      <formula>$A186="barcode"</formula>
+      <formula>OR($A186="audio audit", $A186="text audit", $A186="speed violations count", $A186="speed violations list", $A186="speed violations audit")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q204:W207">
     <cfRule type="expression" dxfId="113" priority="175" stopIfTrue="1">
+      <formula>$A204="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="112" priority="175" stopIfTrue="1">
+      <formula>$A204="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="111" priority="175" stopIfTrue="1">
+      <formula>$A204="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="110" priority="175" stopIfTrue="1">
+      <formula>$A204="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="109" priority="175" stopIfTrue="1">
+      <formula>OR($A204="audio", $A204="video")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="108" priority="175" stopIfTrue="1">
+      <formula>OR($A204="date", $A204="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="107" priority="175" stopIfTrue="1">
+      <formula>$A204="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="106" priority="175" stopIfTrue="1">
+      <formula>$A204="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="105" priority="175" stopIfTrue="1">
+      <formula>$A204="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="104" priority="175" stopIfTrue="1">
+      <formula>$A204="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="103" priority="175" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A204, 16)="select_multiple ", LEN($A204)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A204, 17)))), AND(LEFT($A204, 11)="select_one ", LEN($A204)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A204, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="102" priority="175" stopIfTrue="1">
+      <formula>$A204="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="101" priority="175" stopIfTrue="1">
+      <formula>$A204="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="100" priority="175" stopIfTrue="1">
+      <formula>OR($A204="username", $A204="phonenumber", $A204="start", $A204="end", $A204="deviceid", $A204="subscriberid", $A204="simserial", $A204="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="99" priority="175" stopIfTrue="1">
+      <formula>OR($A204="audio audit", $A204="text audit", $A204="speed violations count", $A204="speed violations list", $A204="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="98" priority="175" stopIfTrue="1">
       <formula>OR($A204="calculate", $A204="calculate_here")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="112" priority="175" stopIfTrue="1">
-      <formula>$A204="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="111" priority="175" stopIfTrue="1">
-      <formula>$A204="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="110" priority="175" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A204, 16)="select_multiple ", LEN($A204)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A204, 17)))), AND(LEFT($A204, 11)="select_one ", LEN($A204)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A204, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="109" priority="175" stopIfTrue="1">
+    <cfRule type="expression" dxfId="97" priority="175" stopIfTrue="1">
       <formula>OR($A204="geopoint", $A204="geoshape", $A204="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="108" priority="175" stopIfTrue="1">
-      <formula>OR($A204="audio audit", $A204="text audit", $A204="speed violations count", $A204="speed violations list", $A204="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="107" priority="175" stopIfTrue="1">
-      <formula>OR($A204="username", $A204="phonenumber", $A204="start", $A204="end", $A204="deviceid", $A204="subscriberid", $A204="simserial", $A204="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="106" priority="175" stopIfTrue="1">
-      <formula>$A204="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="105" priority="175" stopIfTrue="1">
-      <formula>$A204="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="104" priority="175" stopIfTrue="1">
-      <formula>$A204="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="103" priority="175" stopIfTrue="1">
-      <formula>$A204="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="102" priority="175" stopIfTrue="1">
-      <formula>$A204="end repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="101" priority="175" stopIfTrue="1">
-      <formula>OR($A204="audio", $A204="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="100" priority="175" stopIfTrue="1">
-      <formula>OR($A204="date", $A204="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="99" priority="175" stopIfTrue="1">
-      <formula>$A204="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="98" priority="175" stopIfTrue="1">
-      <formula>$A204="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="97" priority="175" stopIfTrue="1">
-      <formula>$A204="note"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q221:W224">
     <cfRule type="expression" dxfId="96" priority="158" stopIfTrue="1">
+      <formula>OR($A221="geopoint", $A221="geoshape", $A221="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="95" priority="158" stopIfTrue="1">
+      <formula>$A221="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="94" priority="158" stopIfTrue="1">
+      <formula>OR($A221="audio audit", $A221="text audit", $A221="speed violations count", $A221="speed violations list", $A221="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="93" priority="158" stopIfTrue="1">
+      <formula>$A221="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="92" priority="158" stopIfTrue="1">
       <formula>OR($A221="calculate", $A221="calculate_here")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="95" priority="158" stopIfTrue="1">
-      <formula>OR($A221="geopoint", $A221="geoshape", $A221="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="94" priority="158" stopIfTrue="1">
+    <cfRule type="expression" dxfId="91" priority="158" stopIfTrue="1">
+      <formula>OR($A221="username", $A221="phonenumber", $A221="start", $A221="end", $A221="deviceid", $A221="subscriberid", $A221="simserial", $A221="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="90" priority="158" stopIfTrue="1">
+      <formula>$A221="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="89" priority="158" stopIfTrue="1">
+      <formula>OR($A221="date", $A221="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="88" priority="158" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A221, 16)="select_multiple ", LEN($A221)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A221, 17)))), AND(LEFT($A221, 11)="select_one ", LEN($A221)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A221, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="87" priority="158" stopIfTrue="1">
+      <formula>$A221="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="86" priority="158" stopIfTrue="1">
+      <formula>$A221="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="85" priority="158" stopIfTrue="1">
+      <formula>$A221="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="84" priority="158" stopIfTrue="1">
+      <formula>$A221="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="83" priority="158" stopIfTrue="1">
+      <formula>$A221="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="82" priority="158" stopIfTrue="1">
+      <formula>OR($A221="audio", $A221="video")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="81" priority="158" stopIfTrue="1">
       <formula>$A221="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="93" priority="158" stopIfTrue="1">
-      <formula>OR($A221="audio", $A221="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="92" priority="158" stopIfTrue="1">
-      <formula>$A221="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="91" priority="158" stopIfTrue="1">
-      <formula>$A221="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="90" priority="158" stopIfTrue="1">
-      <formula>$A221="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="89" priority="158" stopIfTrue="1">
-      <formula>$A221="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="88" priority="158" stopIfTrue="1">
-      <formula>$A221="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="87" priority="158" stopIfTrue="1">
+    <cfRule type="expression" dxfId="80" priority="158" stopIfTrue="1">
       <formula>$A221="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="86" priority="158" stopIfTrue="1">
-      <formula>OR($A221="audio audit", $A221="text audit", $A221="speed violations count", $A221="speed violations list", $A221="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="85" priority="158" stopIfTrue="1">
-      <formula>$A221="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="84" priority="158" stopIfTrue="1">
-      <formula>OR($A221="username", $A221="phonenumber", $A221="start", $A221="end", $A221="deviceid", $A221="subscriberid", $A221="simserial", $A221="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="83" priority="158" stopIfTrue="1">
-      <formula>$A221="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="82" priority="158" stopIfTrue="1">
-      <formula>OR($A221="date", $A221="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="81" priority="158" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A221, 16)="select_multiple ", LEN($A221)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A221, 17)))), AND(LEFT($A221, 11)="select_one ", LEN($A221)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A221, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="80" priority="158" stopIfTrue="1">
-      <formula>$A221="note"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R1:T236">
@@ -17733,46 +17735,46 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:U68 A1:T236 V1:X236 U70:U236">
     <cfRule type="expression" dxfId="76" priority="421" stopIfTrue="1">
-      <formula>$A1="barcode"</formula>
+      <formula>OR($A1="calculate", $A1="calculate_here")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="75" priority="421" stopIfTrue="1">
       <formula>OR($A1="date", $A1="datetime")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="74" priority="421" stopIfTrue="1">
+      <formula>$A1="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="73" priority="421" stopIfTrue="1">
       <formula>OR($A1="audio", $A1="video")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="72" priority="421" stopIfTrue="1">
       <formula>OR($A1="geopoint", $A1="geoshape", $A1="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="72" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="71" priority="421" stopIfTrue="1">
       <formula>OR($A1="audio audit", $A1="text audit", $A1="speed violations count", $A1="speed violations list", $A1="speed violations audit")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="71" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="70" priority="421" stopIfTrue="1">
       <formula>OR($A1="username", $A1="phonenumber", $A1="start", $A1="end", $A1="deviceid", $A1="subscriberid", $A1="simserial", $A1="caseid")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="70" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="69" priority="421" stopIfTrue="1">
       <formula>OR(AND(LEFT($A1, 16)="select_multiple ", LEN($A1)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1, 17)))), AND(LEFT($A1, 11)="select_one ", LEN($A1)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1, 12)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="69" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="68" priority="421" stopIfTrue="1">
       <formula>$A1="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="67" priority="421" stopIfTrue="1">
       <formula>$A1="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="67" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="66" priority="421" stopIfTrue="1">
       <formula>$A1="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="66" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="65" priority="421" stopIfTrue="1">
       <formula>$A1="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="65" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="64" priority="421" stopIfTrue="1">
       <formula>$A1="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="421" stopIfTrue="1">
+    <cfRule type="expression" dxfId="63" priority="421" stopIfTrue="1">
       <formula>$A1="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="63" priority="421" stopIfTrue="1">
-      <formula>OR($A1="calculate", $A1="calculate_here")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U1:U68 D1:D236 O1:O236 U70:U236 V8:V9">
@@ -17906,11 +17908,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W1:W236">
-    <cfRule type="expression" dxfId="22" priority="422">
+    <cfRule type="expression" dxfId="22" priority="422" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1, 14)="sensor_stream ", LEN($A1)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1, 15)))), AND(LEFT($A1, 17)="sensor_statistic ", LEN($A1)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1, 18)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="422">
       <formula>AK1="false"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="21" priority="422" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1, 14)="sensor_stream ", LEN($A1)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1, 15)))), AND(LEFT($A1, 17)="sensor_statistic ", LEN($A1)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1, 18)))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X1:X236">
@@ -17923,43 +17925,43 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="X33:X34">
     <cfRule type="expression" dxfId="18" priority="243" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A33, 16)="select_multiple ", LEN($A33)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A33, 17)))), AND(LEFT($A33, 11)="select_one ", LEN($A33)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A33, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="17" priority="243" stopIfTrue="1">
       <formula>OR($A33="username", $A33="phonenumber", $A33="start", $A33="end", $A33="deviceid", $A33="subscriberid", $A33="simserial", $A33="caseid")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="16" priority="243" stopIfTrue="1">
       <formula>OR($A33="audio audit", $A33="text audit", $A33="speed violations count", $A33="speed violations list", $A33="speed violations audit")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="15" priority="243" stopIfTrue="1">
       <formula>OR($A33="geopoint", $A33="geoshape", $A33="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="243" stopIfTrue="1">
       <formula>$A33="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="243" stopIfTrue="1">
       <formula>$A33="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="243" stopIfTrue="1">
       <formula>OR(AND(LEFT($A33, 14)="sensor_stream ", LEN($A33)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A33, 15)))), AND(LEFT($A33, 17)="sensor_statistic ", LEN($A33)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A33, 18)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="243" stopIfTrue="1">
       <formula>$A33="begin repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="243" stopIfTrue="1">
       <formula>$A33="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="243" stopIfTrue="1">
       <formula>$A33="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="243" stopIfTrue="1">
       <formula>$A33="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="243" stopIfTrue="1">
       <formula>$A33="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="243" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="243" stopIfTrue="1">
       <formula>$A33="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="243" stopIfTrue="1">
-      <formula>$A33="decimal"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="5" priority="243" stopIfTrue="1">
       <formula>OR($A33="calculate", $A33="calculate_here")</formula>
@@ -17977,7 +17979,7 @@
       <formula>$A33="comments"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="243" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A33, 16)="select_multiple ", LEN($A33)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A33, 17)))), AND(LEFT($A33, 11)="select_one ", LEN($A33)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A33, 12)))))</formula>
+      <formula>$A33="decimal"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>